<commit_message>
Actualizacion automatica 06/07/2026 10:10:19.52
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="40" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E32AC8C-2511-47E7-822D-D46509BA8BED}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8C06B202-7D07-4C97-A1C8-F1B3F5624D7D}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$90</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -1179,6 +1182,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:D90"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1216,7 +1220,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1230,7 +1234,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1244,7 +1248,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1258,7 +1262,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1272,7 +1276,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1286,7 +1290,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1300,7 +1304,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1328,7 +1332,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1342,7 +1346,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1356,7 +1360,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1384,7 +1388,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1398,7 +1402,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1412,7 +1416,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1426,7 +1430,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1440,7 +1444,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1454,7 +1458,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1468,7 +1472,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1496,7 +1500,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1510,7 +1514,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1524,7 +1528,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1538,7 +1542,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1552,7 +1556,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1566,7 +1570,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1594,7 +1598,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1608,7 +1612,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1622,7 +1626,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1636,7 +1640,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1650,7 +1654,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1664,7 +1668,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1678,7 +1682,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1706,7 +1710,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1720,7 +1724,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1734,7 +1738,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1748,7 +1752,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="41" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" s="1" customFormat="1" hidden="1" x14ac:dyDescent="0.3">
       <c r="A41" s="1">
         <v>40</v>
       </c>
@@ -1762,7 +1766,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1776,7 +1780,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1804,7 +1808,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1818,7 +1822,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1832,7 +1836,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1846,7 +1850,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1860,7 +1864,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1874,7 +1878,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>50</v>
       </c>
@@ -1888,7 +1892,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>51</v>
       </c>
@@ -1902,7 +1906,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>52</v>
       </c>
@@ -1916,7 +1920,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>53</v>
       </c>
@@ -1930,7 +1934,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>54</v>
       </c>
@@ -1944,7 +1948,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>55</v>
       </c>
@@ -1958,7 +1962,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>56</v>
       </c>
@@ -1972,7 +1976,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>57</v>
       </c>
@@ -1986,7 +1990,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>58</v>
       </c>
@@ -2000,7 +2004,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>59</v>
       </c>
@@ -2014,7 +2018,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>60</v>
       </c>
@@ -2028,7 +2032,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>61</v>
       </c>
@@ -2042,7 +2046,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>62</v>
       </c>
@@ -2056,7 +2060,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>63</v>
       </c>
@@ -2070,7 +2074,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>64</v>
       </c>
@@ -2084,7 +2088,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>65</v>
       </c>
@@ -2098,7 +2102,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>66</v>
       </c>
@@ -2112,7 +2116,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>67</v>
       </c>
@@ -2126,7 +2130,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>68</v>
       </c>
@@ -2140,7 +2144,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>69</v>
       </c>
@@ -2154,7 +2158,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>70</v>
       </c>
@@ -2168,7 +2172,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>71</v>
       </c>
@@ -2182,7 +2186,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>72</v>
       </c>
@@ -2196,7 +2200,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>73</v>
       </c>
@@ -2210,7 +2214,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>74</v>
       </c>
@@ -2224,7 +2228,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>75</v>
       </c>
@@ -2238,7 +2242,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>76</v>
       </c>
@@ -2266,7 +2270,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>78</v>
       </c>
@@ -2280,7 +2284,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>79</v>
       </c>
@@ -2294,7 +2298,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>80</v>
       </c>
@@ -2308,7 +2312,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>81</v>
       </c>
@@ -2322,7 +2326,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>82</v>
       </c>
@@ -2336,7 +2340,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>83</v>
       </c>
@@ -2350,7 +2354,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>84</v>
       </c>
@@ -2364,7 +2368,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>85</v>
       </c>
@@ -2378,7 +2382,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>86</v>
       </c>
@@ -2392,7 +2396,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>87</v>
       </c>
@@ -2406,7 +2410,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>88</v>
       </c>
@@ -2420,7 +2424,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>89</v>
       </c>
@@ -2434,7 +2438,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>90</v>
       </c>
@@ -2449,31 +2453,18 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D90" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="S"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="f031da45812bb81645562bafa3e27792">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="997341155ac57a7f96d45d03b878e5a8" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
@@ -2674,10 +2665,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEA11AD3-ABC0-467F-9346-A4118520785A}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
+    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2694,20 +2716,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEA11AD3-ABC0-467F-9346-A4118520785A}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
-    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica lun 13/07/2026  2:34:21.60
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/02. Encuestas/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="79" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{17D5299C-CFE4-41D6-973E-B374960C5EEE}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C7D8E01-5C67-4889-A419-D07687C46B74}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="119">
   <si>
     <t>CODPER</t>
   </si>
@@ -387,6 +387,12 @@
   </si>
   <si>
     <t>Veronica Aulla Acuña</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>KARIN AYAPI DA SILVA</t>
   </si>
 </sst>
 </file>
@@ -870,9 +876,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -929,10 +934,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1232,7 +1233,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D100"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
@@ -1801,17 +1802,17 @@
         <v>94</v>
       </c>
     </row>
-    <row r="41" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="1">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41">
         <v>40</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" t="s">
         <v>45</v>
       </c>
-      <c r="C41" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D41" s="1" t="s">
+      <c r="C41" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" t="s">
         <v>94</v>
       </c>
     </row>
@@ -2639,6 +2640,20 @@
       </c>
       <c r="D100" t="s">
         <v>115</v>
+      </c>
+    </row>
+    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>117</v>
+      </c>
+      <c r="B101" t="s">
+        <v>118</v>
+      </c>
+      <c r="C101" t="s">
+        <v>7</v>
+      </c>
+      <c r="D101" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>
@@ -2647,12 +2662,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2857,20 +2874,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
+    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2895,12 +2913,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica lun 20/07/2026  9:35:09.88
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/02. Encuestas/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="83" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3C7D8E01-5C67-4889-A419-D07687C46B74}"/>
+  <xr:revisionPtr revIDLastSave="101" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D84A07AA-F4D7-4FDA-9569-CB8DEEF0D4A2}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="125">
   <si>
     <t>CODPER</t>
   </si>
@@ -393,13 +393,31 @@
   </si>
   <si>
     <t>KARIN AYAPI DA SILVA</t>
+  </si>
+  <si>
+    <t>A4</t>
+  </si>
+  <si>
+    <t>KARIN CASTILLO TARAZONA</t>
+  </si>
+  <si>
+    <t>ZULEICKA GUTIERREZ ARAUJO</t>
+  </si>
+  <si>
+    <t>DAVID FIESTAS ROBLES</t>
+  </si>
+  <si>
+    <t>A6</t>
+  </si>
+  <si>
+    <t>A8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -530,6 +548,12 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1233,7 +1257,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:D104"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
@@ -2656,23 +2680,55 @@
         <v>83</v>
       </c>
     </row>
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>119</v>
+      </c>
+      <c r="B102" t="s">
+        <v>120</v>
+      </c>
+      <c r="C102" t="s">
+        <v>7</v>
+      </c>
+      <c r="D102" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>123</v>
+      </c>
+      <c r="B103" t="s">
+        <v>121</v>
+      </c>
+      <c r="C103" t="s">
+        <v>7</v>
+      </c>
+      <c r="D103" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A104" t="s">
+        <v>124</v>
+      </c>
+      <c r="B104" t="s">
+        <v>122</v>
+      </c>
+      <c r="C104" t="s">
+        <v>5</v>
+      </c>
+      <c r="D104" t="s">
+        <v>104</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="f031da45812bb81645562bafa3e27792">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="997341155ac57a7f96d45d03b878e5a8" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
@@ -2873,6 +2929,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -2883,17 +2950,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEA11AD3-ABC0-467F-9346-A4118520785A}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2912,6 +2968,17 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
+    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizacion automatica lun 20/07/2026 11:45:43.11
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/02. Encuestas/Insumos limpieza/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="101" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D84A07AA-F4D7-4FDA-9569-CB8DEEF0D4A2}"/>
+  <xr:revisionPtr revIDLastSave="126" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A2B603C-7132-40E7-BCB7-32B83FDCD1C3}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,9 @@
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$90</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$104</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="123">
   <si>
     <t>CODPER</t>
   </si>
@@ -230,13 +230,7 @@
     <t xml:space="preserve">ALISON VICTORIA CAJAHUARINGA CUEVA                                              </t>
   </si>
   <si>
-    <t xml:space="preserve">APURIMAC                                          </t>
-  </si>
-  <si>
     <t xml:space="preserve">ELIZABETH LOZANO VARGAS                                                         </t>
-  </si>
-  <si>
-    <t xml:space="preserve">HUANUCO                                           </t>
   </si>
   <si>
     <t xml:space="preserve">FLOR NOEMI EUGENIO LUNA                                                         </t>
@@ -1291,7 +1285,7 @@
         <v>5</v>
       </c>
       <c r="D2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
@@ -1305,7 +1299,7 @@
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
@@ -1319,7 +1313,7 @@
         <v>7</v>
       </c>
       <c r="D4" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
@@ -1333,7 +1327,7 @@
         <v>7</v>
       </c>
       <c r="D5" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
@@ -1347,7 +1341,7 @@
         <v>7</v>
       </c>
       <c r="D6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
@@ -1361,7 +1355,7 @@
         <v>7</v>
       </c>
       <c r="D7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
@@ -1375,7 +1369,7 @@
         <v>7</v>
       </c>
       <c r="D8" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
@@ -1389,7 +1383,7 @@
         <v>7</v>
       </c>
       <c r="D9" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.3">
@@ -1403,7 +1397,7 @@
         <v>5</v>
       </c>
       <c r="D10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
@@ -1417,7 +1411,7 @@
         <v>7</v>
       </c>
       <c r="D11" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
@@ -1431,7 +1425,7 @@
         <v>7</v>
       </c>
       <c r="D12" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
@@ -1445,7 +1439,7 @@
         <v>7</v>
       </c>
       <c r="D13" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.3">
@@ -1459,7 +1453,7 @@
         <v>5</v>
       </c>
       <c r="D14" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
@@ -1473,7 +1467,7 @@
         <v>7</v>
       </c>
       <c r="D15" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
@@ -1487,7 +1481,7 @@
         <v>7</v>
       </c>
       <c r="D16" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
@@ -1501,7 +1495,7 @@
         <v>7</v>
       </c>
       <c r="D17" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
@@ -1515,7 +1509,7 @@
         <v>7</v>
       </c>
       <c r="D18" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
@@ -1529,7 +1523,7 @@
         <v>7</v>
       </c>
       <c r="D19" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
@@ -1543,7 +1537,7 @@
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
@@ -1557,7 +1551,7 @@
         <v>7</v>
       </c>
       <c r="D21" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
@@ -1571,7 +1565,7 @@
         <v>5</v>
       </c>
       <c r="D22" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
@@ -1585,7 +1579,7 @@
         <v>7</v>
       </c>
       <c r="D23" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
@@ -1599,7 +1593,7 @@
         <v>7</v>
       </c>
       <c r="D24" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
@@ -1613,7 +1607,7 @@
         <v>7</v>
       </c>
       <c r="D25" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
@@ -1627,7 +1621,7 @@
         <v>7</v>
       </c>
       <c r="D26" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
@@ -1641,7 +1635,7 @@
         <v>7</v>
       </c>
       <c r="D27" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
@@ -1655,7 +1649,7 @@
         <v>7</v>
       </c>
       <c r="D28" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
@@ -1669,7 +1663,7 @@
         <v>5</v>
       </c>
       <c r="D29" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.3">
@@ -1683,7 +1677,7 @@
         <v>7</v>
       </c>
       <c r="D30" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.3">
@@ -1697,7 +1691,7 @@
         <v>7</v>
       </c>
       <c r="D31" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
@@ -1711,7 +1705,7 @@
         <v>7</v>
       </c>
       <c r="D32" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.3">
@@ -1725,7 +1719,7 @@
         <v>7</v>
       </c>
       <c r="D33" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.3">
@@ -1739,7 +1733,7 @@
         <v>7</v>
       </c>
       <c r="D34" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
@@ -1753,7 +1747,7 @@
         <v>7</v>
       </c>
       <c r="D35" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.3">
@@ -1767,7 +1761,7 @@
         <v>7</v>
       </c>
       <c r="D36" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.3">
@@ -1781,7 +1775,7 @@
         <v>5</v>
       </c>
       <c r="D37" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
@@ -1795,7 +1789,7 @@
         <v>7</v>
       </c>
       <c r="D38" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
@@ -1809,7 +1803,7 @@
         <v>7</v>
       </c>
       <c r="D39" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
@@ -1823,7 +1817,7 @@
         <v>7</v>
       </c>
       <c r="D40" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
@@ -1837,7 +1831,7 @@
         <v>7</v>
       </c>
       <c r="D41" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
@@ -1851,7 +1845,7 @@
         <v>7</v>
       </c>
       <c r="D42" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
@@ -1865,7 +1859,7 @@
         <v>7</v>
       </c>
       <c r="D43" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.3">
@@ -1879,7 +1873,7 @@
         <v>5</v>
       </c>
       <c r="D44" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.3">
@@ -1893,7 +1887,7 @@
         <v>7</v>
       </c>
       <c r="D45" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.3">
@@ -1907,7 +1901,7 @@
         <v>7</v>
       </c>
       <c r="D46" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
@@ -1921,7 +1915,7 @@
         <v>7</v>
       </c>
       <c r="D47" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.3">
@@ -1935,7 +1929,7 @@
         <v>7</v>
       </c>
       <c r="D48" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="49" spans="1:4" x14ac:dyDescent="0.3">
@@ -1949,7 +1943,7 @@
         <v>7</v>
       </c>
       <c r="D49" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="50" spans="1:4" x14ac:dyDescent="0.3">
@@ -1963,7 +1957,7 @@
         <v>7</v>
       </c>
       <c r="D50" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="51" spans="1:4" x14ac:dyDescent="0.3">
@@ -1977,7 +1971,7 @@
         <v>7</v>
       </c>
       <c r="D51" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="52" spans="1:4" x14ac:dyDescent="0.3">
@@ -1991,7 +1985,7 @@
         <v>7</v>
       </c>
       <c r="D52" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="53" spans="1:4" x14ac:dyDescent="0.3">
@@ -2005,7 +1999,7 @@
         <v>7</v>
       </c>
       <c r="D53" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="54" spans="1:4" x14ac:dyDescent="0.3">
@@ -2019,7 +2013,7 @@
         <v>7</v>
       </c>
       <c r="D54" t="s">
-        <v>66</v>
+        <v>93</v>
       </c>
     </row>
     <row r="55" spans="1:4" x14ac:dyDescent="0.3">
@@ -2033,7 +2027,7 @@
         <v>7</v>
       </c>
       <c r="D55" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
@@ -2047,7 +2041,7 @@
         <v>7</v>
       </c>
       <c r="D56" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="57" spans="1:4" x14ac:dyDescent="0.3">
@@ -2061,7 +2055,7 @@
         <v>7</v>
       </c>
       <c r="D57" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
@@ -2075,7 +2069,7 @@
         <v>7</v>
       </c>
       <c r="D58" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
@@ -2089,7 +2083,7 @@
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
@@ -2097,13 +2091,13 @@
         <v>60</v>
       </c>
       <c r="B60" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C60" t="s">
         <v>7</v>
       </c>
       <c r="D60" t="s">
-        <v>66</v>
+        <v>93</v>
       </c>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.3">
@@ -2111,13 +2105,13 @@
         <v>61</v>
       </c>
       <c r="B61" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C61" t="s">
         <v>7</v>
       </c>
       <c r="D61" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
@@ -2125,13 +2119,13 @@
         <v>62</v>
       </c>
       <c r="B62" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C62" t="s">
         <v>7</v>
       </c>
       <c r="D62" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
@@ -2139,13 +2133,13 @@
         <v>63</v>
       </c>
       <c r="B63" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C63" t="s">
         <v>7</v>
       </c>
       <c r="D63" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
@@ -2153,13 +2147,13 @@
         <v>64</v>
       </c>
       <c r="B64" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C64" t="s">
         <v>7</v>
       </c>
       <c r="D64" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
@@ -2167,13 +2161,13 @@
         <v>65</v>
       </c>
       <c r="B65" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C65" t="s">
         <v>7</v>
       </c>
       <c r="D65" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
@@ -2187,7 +2181,7 @@
         <v>7</v>
       </c>
       <c r="D66" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
@@ -2195,13 +2189,13 @@
         <v>67</v>
       </c>
       <c r="B67" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C67" t="s">
         <v>7</v>
       </c>
       <c r="D67" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
@@ -2209,13 +2203,13 @@
         <v>68</v>
       </c>
       <c r="B68" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C68" t="s">
         <v>7</v>
       </c>
       <c r="D68" t="s">
-        <v>64</v>
+        <v>91</v>
       </c>
     </row>
     <row r="69" spans="1:4" x14ac:dyDescent="0.3">
@@ -2223,13 +2217,13 @@
         <v>69</v>
       </c>
       <c r="B69" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C69" t="s">
         <v>7</v>
       </c>
       <c r="D69" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="70" spans="1:4" x14ac:dyDescent="0.3">
@@ -2237,13 +2231,13 @@
         <v>70</v>
       </c>
       <c r="B70" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C70" t="s">
         <v>7</v>
       </c>
       <c r="D70" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="71" spans="1:4" x14ac:dyDescent="0.3">
@@ -2251,13 +2245,13 @@
         <v>71</v>
       </c>
       <c r="B71" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="C71" t="s">
         <v>7</v>
       </c>
       <c r="D71" t="s">
-        <v>66</v>
+        <v>93</v>
       </c>
     </row>
     <row r="72" spans="1:4" x14ac:dyDescent="0.3">
@@ -2265,13 +2259,13 @@
         <v>72</v>
       </c>
       <c r="B72" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C72" t="s">
         <v>7</v>
       </c>
       <c r="D72" t="s">
-        <v>66</v>
+        <v>93</v>
       </c>
     </row>
     <row r="73" spans="1:4" x14ac:dyDescent="0.3">
@@ -2279,13 +2273,13 @@
         <v>73</v>
       </c>
       <c r="B73" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C73" t="s">
         <v>7</v>
       </c>
       <c r="D73" t="s">
-        <v>66</v>
+        <v>93</v>
       </c>
     </row>
     <row r="74" spans="1:4" x14ac:dyDescent="0.3">
@@ -2293,13 +2287,13 @@
         <v>74</v>
       </c>
       <c r="B74" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C74" t="s">
         <v>7</v>
       </c>
       <c r="D74" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="75" spans="1:4" x14ac:dyDescent="0.3">
@@ -2307,13 +2301,13 @@
         <v>75</v>
       </c>
       <c r="B75" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C75" t="s">
         <v>7</v>
       </c>
       <c r="D75" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
@@ -2321,13 +2315,13 @@
         <v>76</v>
       </c>
       <c r="B76" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C76" t="s">
         <v>7</v>
       </c>
       <c r="D76" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="77" spans="1:4" x14ac:dyDescent="0.3">
@@ -2335,13 +2329,13 @@
         <v>77</v>
       </c>
       <c r="B77" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C77" t="s">
         <v>5</v>
       </c>
       <c r="D77" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="78" spans="1:4" x14ac:dyDescent="0.3">
@@ -2349,13 +2343,13 @@
         <v>78</v>
       </c>
       <c r="B78" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C78" t="s">
         <v>7</v>
       </c>
       <c r="D78" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="79" spans="1:4" x14ac:dyDescent="0.3">
@@ -2363,13 +2357,13 @@
         <v>79</v>
       </c>
       <c r="B79" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C79" t="s">
         <v>7</v>
       </c>
       <c r="D79" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="80" spans="1:4" x14ac:dyDescent="0.3">
@@ -2377,13 +2371,13 @@
         <v>80</v>
       </c>
       <c r="B80" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C80" t="s">
         <v>7</v>
       </c>
       <c r="D80" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
@@ -2391,13 +2385,13 @@
         <v>81</v>
       </c>
       <c r="B81" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C81" t="s">
         <v>7</v>
       </c>
       <c r="D81" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
@@ -2405,13 +2399,13 @@
         <v>82</v>
       </c>
       <c r="B82" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C82" t="s">
         <v>7</v>
       </c>
       <c r="D82" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
@@ -2419,13 +2413,13 @@
         <v>83</v>
       </c>
       <c r="B83" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C83" t="s">
         <v>7</v>
       </c>
       <c r="D83" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
@@ -2433,13 +2427,13 @@
         <v>84</v>
       </c>
       <c r="B84" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C84" t="s">
         <v>7</v>
       </c>
       <c r="D84" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
@@ -2447,13 +2441,13 @@
         <v>85</v>
       </c>
       <c r="B85" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C85" t="s">
         <v>7</v>
       </c>
       <c r="D85" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
@@ -2461,13 +2455,13 @@
         <v>86</v>
       </c>
       <c r="B86" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C86" t="s">
         <v>7</v>
       </c>
       <c r="D86" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
@@ -2475,13 +2469,13 @@
         <v>87</v>
       </c>
       <c r="B87" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C87" t="s">
         <v>7</v>
       </c>
       <c r="D87" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
@@ -2489,13 +2483,13 @@
         <v>88</v>
       </c>
       <c r="B88" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C88" t="s">
         <v>7</v>
       </c>
       <c r="D88" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.3">
@@ -2503,13 +2497,13 @@
         <v>89</v>
       </c>
       <c r="B89" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C89" t="s">
         <v>7</v>
       </c>
       <c r="D89" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.3">
@@ -2517,13 +2511,13 @@
         <v>90</v>
       </c>
       <c r="B90" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C90" t="s">
         <v>7</v>
       </c>
       <c r="D90" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
@@ -2531,13 +2525,13 @@
         <v>91</v>
       </c>
       <c r="B91" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C91" t="s">
         <v>7</v>
       </c>
       <c r="D91" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.3">
@@ -2545,13 +2539,13 @@
         <v>92</v>
       </c>
       <c r="B92" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C92" t="s">
         <v>5</v>
       </c>
       <c r="D92" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
@@ -2559,13 +2553,13 @@
         <v>93</v>
       </c>
       <c r="B93" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C93" t="s">
         <v>7</v>
       </c>
       <c r="D93" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
@@ -2573,13 +2567,13 @@
         <v>94</v>
       </c>
       <c r="B94" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C94" t="s">
         <v>7</v>
       </c>
       <c r="D94" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
@@ -2587,13 +2581,13 @@
         <v>95</v>
       </c>
       <c r="B95" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C95" t="s">
         <v>7</v>
       </c>
       <c r="D95" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
@@ -2601,13 +2595,13 @@
         <v>96</v>
       </c>
       <c r="B96" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C96" t="s">
         <v>7</v>
       </c>
       <c r="D96" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.3">
@@ -2615,13 +2609,13 @@
         <v>97</v>
       </c>
       <c r="B97" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C97" t="s">
         <v>7</v>
       </c>
       <c r="D97" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="98" spans="1:4" x14ac:dyDescent="0.3">
@@ -2629,13 +2623,13 @@
         <v>98</v>
       </c>
       <c r="B98" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C98" t="s">
         <v>7</v>
       </c>
       <c r="D98" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.3">
@@ -2643,83 +2637,83 @@
         <v>99</v>
       </c>
       <c r="B99" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C99" t="s">
         <v>7</v>
       </c>
       <c r="D99" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B100" t="s">
+        <v>111</v>
+      </c>
+      <c r="C100" t="s">
+        <v>7</v>
+      </c>
+      <c r="D100" t="s">
         <v>113</v>
-      </c>
-      <c r="C100" t="s">
-        <v>7</v>
-      </c>
-      <c r="D100" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B101" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C101" t="s">
         <v>7</v>
       </c>
       <c r="D101" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B102" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C102" t="s">
         <v>7</v>
       </c>
       <c r="D102" t="s">
-        <v>104</v>
+        <v>84</v>
       </c>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B103" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C103" t="s">
         <v>7</v>
       </c>
       <c r="D103" t="s">
-        <v>104</v>
+        <v>84</v>
       </c>
     </row>
     <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="B104" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C104" t="s">
         <v>5</v>
       </c>
       <c r="D104" t="s">
-        <v>104</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -2729,8 +2723,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="12" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="f031da45812bb81645562bafa3e27792">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="997341155ac57a7f96d45d03b878e5a8" ns2:_="" ns3:_="">
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="07c8fde6007faf37af3ccef690656753">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1f83a7a0bc9c2dabcf9590cf8de720c" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
     <xsd:import namespace="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
     <xsd:element name="properties">
@@ -2750,6 +2753,7 @@
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -2812,6 +2816,11 @@
     <xsd:element name="MediaLengthInSeconds" ma:index="19" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="20" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -2929,7 +2938,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
@@ -2940,17 +2949,16 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EEA11AD3-ABC0-467F-9346-A4118520785A}">
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97189664-1794-4876-AECF-20AF585E9009}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
@@ -2968,7 +2976,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2977,12 +2985,4 @@
     <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica mar 21/07/2026  9:48:14.11
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -5,20 +5,20 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/02. Encuestas/Insumos limpieza/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="126" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A2B603C-7132-40E7-BCB7-32B83FDCD1C3}"/>
+  <xr:revisionPtr revIDLastSave="151" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A3D3713-BF73-4B16-8F19-31D5F8377808}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$107</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="139">
   <si>
     <t>CODPER</t>
   </si>
@@ -405,6 +405,54 @@
   </si>
   <si>
     <t>A8</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>A3</t>
+  </si>
+  <si>
+    <t>A5</t>
+  </si>
+  <si>
+    <t>A9</t>
+  </si>
+  <si>
+    <t>B0</t>
+  </si>
+  <si>
+    <t>B1</t>
+  </si>
+  <si>
+    <t>B2</t>
+  </si>
+  <si>
+    <t>B3</t>
+  </si>
+  <si>
+    <t>CATHERINE DAMIAN HUAMAYALLI</t>
+  </si>
+  <si>
+    <t>MILAGROS HENRIQUEZ CALLIRGOS</t>
+  </si>
+  <si>
+    <t>MARIA DEL ROCIO BURGA ROJAS</t>
+  </si>
+  <si>
+    <t>ROXANA GADEA</t>
+  </si>
+  <si>
+    <t>YOVANNA CASAS</t>
+  </si>
+  <si>
+    <t>LAURA ZAPATA POEMAPE</t>
+  </si>
+  <si>
+    <t>EDITH MAURICIO GRIJALVA</t>
+  </si>
+  <si>
+    <t>MONICA POZO LOZANO</t>
   </si>
 </sst>
 </file>
@@ -1251,16 +1299,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D104"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D112"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="58.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="38.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1274,7 +1322,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1288,7 +1336,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1302,7 +1350,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1316,7 +1364,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1330,7 +1378,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1344,7 +1392,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1358,7 +1406,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1372,7 +1420,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1386,7 +1434,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1400,7 +1448,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1414,7 +1462,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1428,7 +1476,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1442,7 +1490,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1456,7 +1504,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1470,7 +1518,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1484,7 +1532,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1498,7 +1546,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1512,7 +1560,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1526,7 +1574,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1540,7 +1588,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1554,7 +1602,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1568,7 +1616,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1582,7 +1630,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1596,7 +1644,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1610,7 +1658,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1624,7 +1672,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1638,7 +1686,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1652,7 +1700,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1666,7 +1714,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1680,7 +1728,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1694,7 +1742,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1708,7 +1756,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1722,7 +1770,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1736,7 +1784,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1750,7 +1798,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1764,7 +1812,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1778,7 +1826,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1792,7 +1840,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1806,7 +1854,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1820,7 +1868,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1834,7 +1882,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1848,7 +1896,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1862,7 +1910,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1876,7 +1924,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1890,7 +1938,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1904,7 +1952,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1918,7 +1966,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1932,7 +1980,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1946,7 +1994,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>50</v>
       </c>
@@ -1960,7 +2008,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>51</v>
       </c>
@@ -1974,7 +2022,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>52</v>
       </c>
@@ -1988,7 +2036,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>53</v>
       </c>
@@ -2002,7 +2050,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>54</v>
       </c>
@@ -2016,7 +2064,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>55</v>
       </c>
@@ -2030,7 +2078,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>56</v>
       </c>
@@ -2044,7 +2092,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>57</v>
       </c>
@@ -2058,7 +2106,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>58</v>
       </c>
@@ -2072,7 +2120,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>59</v>
       </c>
@@ -2086,7 +2134,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>60</v>
       </c>
@@ -2100,7 +2148,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>61</v>
       </c>
@@ -2114,7 +2162,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>62</v>
       </c>
@@ -2128,7 +2176,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>63</v>
       </c>
@@ -2142,7 +2190,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>64</v>
       </c>
@@ -2156,7 +2204,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>65</v>
       </c>
@@ -2170,7 +2218,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>66</v>
       </c>
@@ -2184,7 +2232,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>67</v>
       </c>
@@ -2198,7 +2246,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>68</v>
       </c>
@@ -2212,7 +2260,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>69</v>
       </c>
@@ -2226,7 +2274,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>70</v>
       </c>
@@ -2240,7 +2288,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>71</v>
       </c>
@@ -2254,7 +2302,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>72</v>
       </c>
@@ -2268,7 +2316,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>73</v>
       </c>
@@ -2282,7 +2330,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>74</v>
       </c>
@@ -2296,7 +2344,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>75</v>
       </c>
@@ -2310,7 +2358,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>76</v>
       </c>
@@ -2324,7 +2372,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>77</v>
       </c>
@@ -2338,7 +2386,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>78</v>
       </c>
@@ -2352,7 +2400,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>79</v>
       </c>
@@ -2366,7 +2414,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>80</v>
       </c>
@@ -2380,7 +2428,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>81</v>
       </c>
@@ -2394,7 +2442,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>82</v>
       </c>
@@ -2408,7 +2456,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>83</v>
       </c>
@@ -2422,7 +2470,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>84</v>
       </c>
@@ -2436,7 +2484,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>85</v>
       </c>
@@ -2450,7 +2498,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>86</v>
       </c>
@@ -2464,7 +2512,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>87</v>
       </c>
@@ -2478,7 +2526,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>88</v>
       </c>
@@ -2492,7 +2540,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>89</v>
       </c>
@@ -2506,7 +2554,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>90</v>
       </c>
@@ -2520,7 +2568,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>91</v>
       </c>
@@ -2534,7 +2582,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>92</v>
       </c>
@@ -2548,7 +2596,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>93</v>
       </c>
@@ -2562,7 +2610,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>94</v>
       </c>
@@ -2576,7 +2624,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>95</v>
       </c>
@@ -2590,7 +2638,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>96</v>
       </c>
@@ -2604,7 +2652,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>97</v>
       </c>
@@ -2618,7 +2666,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>98</v>
       </c>
@@ -2632,7 +2680,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>99</v>
       </c>
@@ -2646,7 +2694,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>112</v>
       </c>
@@ -2660,7 +2708,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>115</v>
       </c>
@@ -2674,12 +2722,12 @@
         <v>81</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B102" t="s">
-        <v>118</v>
+        <v>131</v>
       </c>
       <c r="C102" t="s">
         <v>7</v>
@@ -2688,12 +2736,12 @@
         <v>84</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B103" t="s">
-        <v>119</v>
+        <v>132</v>
       </c>
       <c r="C103" t="s">
         <v>7</v>
@@ -2702,17 +2750,129 @@
         <v>84</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
+        <v>117</v>
+      </c>
+      <c r="B104" t="s">
+        <v>118</v>
+      </c>
+      <c r="C104" t="s">
+        <v>7</v>
+      </c>
+      <c r="D104" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>125</v>
+      </c>
+      <c r="B105" t="s">
+        <v>133</v>
+      </c>
+      <c r="C105" t="s">
+        <v>7</v>
+      </c>
+      <c r="D105" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>121</v>
+      </c>
+      <c r="B106" t="s">
+        <v>119</v>
+      </c>
+      <c r="C106" t="s">
+        <v>7</v>
+      </c>
+      <c r="D106" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
         <v>122</v>
       </c>
-      <c r="B104" t="s">
+      <c r="B107" t="s">
         <v>120</v>
       </c>
-      <c r="C104" t="s">
+      <c r="C107" t="s">
         <v>5</v>
       </c>
-      <c r="D104" t="s">
+      <c r="D107" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>126</v>
+      </c>
+      <c r="B108" t="s">
+        <v>134</v>
+      </c>
+      <c r="C108" t="s">
+        <v>7</v>
+      </c>
+      <c r="D108" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>127</v>
+      </c>
+      <c r="B109" t="s">
+        <v>135</v>
+      </c>
+      <c r="C109" t="s">
+        <v>7</v>
+      </c>
+      <c r="D109" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>128</v>
+      </c>
+      <c r="B110" t="s">
+        <v>136</v>
+      </c>
+      <c r="C110" t="s">
+        <v>7</v>
+      </c>
+      <c r="D110" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>129</v>
+      </c>
+      <c r="B111" t="s">
+        <v>137</v>
+      </c>
+      <c r="C111" t="s">
+        <v>7</v>
+      </c>
+      <c r="D111" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>130</v>
+      </c>
+      <c r="B112" t="s">
+        <v>138</v>
+      </c>
+      <c r="C112" t="s">
+        <v>7</v>
+      </c>
+      <c r="D112" t="s">
         <v>84</v>
       </c>
     </row>
@@ -2723,12 +2883,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2939,20 +3101,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
+    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2977,12 +3140,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica mié 22/07/2026 10:03:36.87
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="151" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A3D3713-BF73-4B16-8F19-31D5F8377808}"/>
+  <xr:revisionPtr revIDLastSave="155" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2A9FEE7-B318-4828-B1BF-D13C51ABB45D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$107</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$112</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1300,15 +1300,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D112"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="58.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="4.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="38.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="58.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1336,7 +1336,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1350,7 +1350,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1364,7 +1364,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1392,7 +1392,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1406,7 +1406,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1420,7 +1420,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1434,7 +1434,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1476,7 +1476,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1490,7 +1490,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1504,7 +1504,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1518,7 +1518,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1532,7 +1532,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1546,7 +1546,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1560,7 +1560,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1574,7 +1574,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1588,7 +1588,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1602,7 +1602,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1616,7 +1616,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1644,7 +1644,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1658,7 +1658,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1672,7 +1672,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1700,7 +1700,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1714,7 +1714,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1728,7 +1728,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1742,7 +1742,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1756,7 +1756,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1770,7 +1770,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1798,7 +1798,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1812,7 +1812,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1840,7 +1840,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1854,7 +1854,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1868,7 +1868,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1882,7 +1882,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1910,7 +1910,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1924,7 +1924,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1938,7 +1938,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1952,7 +1952,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1966,7 +1966,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1980,7 +1980,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1994,7 +1994,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>50</v>
       </c>
@@ -2008,7 +2008,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>51</v>
       </c>
@@ -2022,7 +2022,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>52</v>
       </c>
@@ -2036,7 +2036,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>53</v>
       </c>
@@ -2050,7 +2050,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>54</v>
       </c>
@@ -2064,7 +2064,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>55</v>
       </c>
@@ -2078,7 +2078,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>56</v>
       </c>
@@ -2092,7 +2092,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>57</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>58</v>
       </c>
@@ -2120,7 +2120,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>59</v>
       </c>
@@ -2134,7 +2134,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>60</v>
       </c>
@@ -2148,7 +2148,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>61</v>
       </c>
@@ -2162,7 +2162,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>62</v>
       </c>
@@ -2176,7 +2176,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>63</v>
       </c>
@@ -2190,7 +2190,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>64</v>
       </c>
@@ -2204,7 +2204,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>65</v>
       </c>
@@ -2218,7 +2218,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>66</v>
       </c>
@@ -2232,7 +2232,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>67</v>
       </c>
@@ -2246,7 +2246,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>68</v>
       </c>
@@ -2260,7 +2260,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>69</v>
       </c>
@@ -2274,7 +2274,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>70</v>
       </c>
@@ -2288,7 +2288,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>71</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>72</v>
       </c>
@@ -2316,7 +2316,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>73</v>
       </c>
@@ -2330,7 +2330,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>74</v>
       </c>
@@ -2344,7 +2344,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>75</v>
       </c>
@@ -2358,7 +2358,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>76</v>
       </c>
@@ -2372,7 +2372,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>77</v>
       </c>
@@ -2386,7 +2386,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>78</v>
       </c>
@@ -2400,7 +2400,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>79</v>
       </c>
@@ -2414,7 +2414,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>80</v>
       </c>
@@ -2428,7 +2428,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>81</v>
       </c>
@@ -2442,7 +2442,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>82</v>
       </c>
@@ -2456,7 +2456,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>83</v>
       </c>
@@ -2470,7 +2470,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>84</v>
       </c>
@@ -2484,7 +2484,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>85</v>
       </c>
@@ -2498,7 +2498,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>86</v>
       </c>
@@ -2512,7 +2512,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>87</v>
       </c>
@@ -2526,7 +2526,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>88</v>
       </c>
@@ -2540,7 +2540,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>89</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>90</v>
       </c>
@@ -2568,7 +2568,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>91</v>
       </c>
@@ -2582,7 +2582,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>92</v>
       </c>
@@ -2596,7 +2596,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>93</v>
       </c>
@@ -2610,7 +2610,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>94</v>
       </c>
@@ -2624,7 +2624,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>95</v>
       </c>
@@ -2638,7 +2638,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>96</v>
       </c>
@@ -2652,7 +2652,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>97</v>
       </c>
@@ -2666,7 +2666,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>98</v>
       </c>
@@ -2677,10 +2677,10 @@
         <v>7</v>
       </c>
       <c r="D98" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.25">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>99</v>
       </c>
@@ -2694,7 +2694,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>112</v>
       </c>
@@ -2708,7 +2708,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>115</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>123</v>
       </c>
@@ -2736,7 +2736,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>124</v>
       </c>
@@ -2750,7 +2750,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>117</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>125</v>
       </c>
@@ -2778,7 +2778,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>121</v>
       </c>
@@ -2792,7 +2792,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>122</v>
       </c>
@@ -2806,7 +2806,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>126</v>
       </c>
@@ -2820,7 +2820,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>127</v>
       </c>
@@ -2834,7 +2834,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>128</v>
       </c>
@@ -2848,7 +2848,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>129</v>
       </c>
@@ -2862,7 +2862,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>130</v>
       </c>

</xml_diff>

<commit_message>
Actualizacion automatica jue 30/07/2026  9:46:52.14
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="155" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A2A9FEE7-B318-4828-B1BF-D13C51ABB45D}"/>
+  <xr:revisionPtr revIDLastSave="163" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C6D0910-94C6-426F-A3D0-6267272AD9D5}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$112</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1299,6 +1299,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:D112"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1322,7 +1323,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1336,7 +1337,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1350,7 +1351,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1364,7 +1365,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1378,7 +1379,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1392,7 +1393,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1406,7 +1407,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1420,7 +1421,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1434,7 +1435,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1448,7 +1449,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1462,7 +1463,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1476,7 +1477,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1490,7 +1491,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1506,10 +1507,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>63</v>
       </c>
       <c r="C15" t="s">
         <v>7</v>
@@ -1520,10 +1521,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>63</v>
       </c>
       <c r="C16" t="s">
         <v>7</v>
@@ -1534,24 +1535,24 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>16</v>
+        <v>65</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>70</v>
       </c>
       <c r="C17" t="s">
         <v>7</v>
       </c>
       <c r="D17" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>17</v>
+        <v>68</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>72</v>
       </c>
       <c r="C18" t="s">
         <v>7</v>
@@ -1562,38 +1563,38 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>18</v>
+        <v>83</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>94</v>
       </c>
       <c r="C19" t="s">
         <v>7</v>
       </c>
       <c r="D19" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>43</v>
       </c>
       <c r="C20" t="s">
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="B21" t="s">
-        <v>25</v>
+        <v>71</v>
       </c>
       <c r="C21" t="s">
         <v>7</v>
@@ -1602,7 +1603,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1616,7 +1617,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1630,7 +1631,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1644,7 +1645,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1658,7 +1659,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1672,7 +1673,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1686,7 +1687,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1700,7 +1701,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1714,7 +1715,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1728,7 +1729,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1742,7 +1743,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1756,7 +1757,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1770,7 +1771,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1784,7 +1785,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1798,7 +1799,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1812,7 +1813,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1828,52 +1829,52 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38">
-        <v>37</v>
+        <v>17</v>
       </c>
       <c r="B38" t="s">
-        <v>42</v>
+        <v>22</v>
       </c>
       <c r="C38" t="s">
         <v>7</v>
       </c>
       <c r="D38" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>38</v>
+        <v>14</v>
       </c>
       <c r="B39" t="s">
-        <v>43</v>
+        <v>19</v>
       </c>
       <c r="C39" t="s">
         <v>7</v>
       </c>
       <c r="D39" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="B40" t="s">
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="C40" t="s">
         <v>7</v>
       </c>
       <c r="D40" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B41" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C41" t="s">
         <v>7</v>
@@ -1884,33 +1885,33 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="B42" t="s">
-        <v>46</v>
+        <v>20</v>
       </c>
       <c r="C42" t="s">
         <v>7</v>
       </c>
       <c r="D42" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="B43" t="s">
-        <v>47</v>
+        <v>21</v>
       </c>
       <c r="C43" t="s">
         <v>7</v>
       </c>
       <c r="D43" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1924,7 +1925,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1938,7 +1939,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1952,7 +1953,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1966,7 +1967,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1980,7 +1981,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1994,7 +1995,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>50</v>
       </c>
@@ -2008,7 +2009,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>51</v>
       </c>
@@ -2022,7 +2023,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>52</v>
       </c>
@@ -2036,7 +2037,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>53</v>
       </c>
@@ -2050,7 +2051,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>54</v>
       </c>
@@ -2064,7 +2065,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>55</v>
       </c>
@@ -2078,7 +2079,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>56</v>
       </c>
@@ -2092,7 +2093,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>57</v>
       </c>
@@ -2106,7 +2107,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>58</v>
       </c>
@@ -2122,19 +2123,19 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="B59" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C59" t="s">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>60</v>
       </c>
@@ -2148,7 +2149,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>61</v>
       </c>
@@ -2164,24 +2165,24 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>62</v>
+        <v>20</v>
       </c>
       <c r="B62" t="s">
-        <v>67</v>
+        <v>25</v>
       </c>
       <c r="C62" t="s">
         <v>7</v>
       </c>
       <c r="D62" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="B63" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="C63" t="s">
         <v>7</v>
@@ -2206,10 +2207,10 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65">
-        <v>65</v>
+        <v>84</v>
       </c>
       <c r="B65" t="s">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="C65" t="s">
         <v>7</v>
@@ -2220,38 +2221,38 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="B66" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C66" t="s">
         <v>7</v>
       </c>
       <c r="D66" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67">
-        <v>67</v>
+        <v>39</v>
       </c>
       <c r="B67" t="s">
-        <v>71</v>
+        <v>44</v>
       </c>
       <c r="C67" t="s">
         <v>7</v>
       </c>
       <c r="D67" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>68</v>
+        <v>18</v>
       </c>
       <c r="B68" t="s">
-        <v>72</v>
+        <v>23</v>
       </c>
       <c r="C68" t="s">
         <v>7</v>
@@ -2260,7 +2261,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>69</v>
       </c>
@@ -2274,7 +2275,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>70</v>
       </c>
@@ -2288,7 +2289,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>71</v>
       </c>
@@ -2302,7 +2303,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>72</v>
       </c>
@@ -2316,7 +2317,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>73</v>
       </c>
@@ -2330,7 +2331,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>74</v>
       </c>
@@ -2344,7 +2345,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>75</v>
       </c>
@@ -2358,7 +2359,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>76</v>
       </c>
@@ -2372,7 +2373,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>77</v>
       </c>
@@ -2386,7 +2387,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>78</v>
       </c>
@@ -2400,7 +2401,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>79</v>
       </c>
@@ -2414,7 +2415,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>80</v>
       </c>
@@ -2428,7 +2429,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>81</v>
       </c>
@@ -2442,7 +2443,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>82</v>
       </c>
@@ -2458,10 +2459,10 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="B83" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="C83" t="s">
         <v>7</v>
@@ -2472,10 +2473,10 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84">
-        <v>84</v>
+        <v>37</v>
       </c>
       <c r="B84" t="s">
-        <v>95</v>
+        <v>42</v>
       </c>
       <c r="C84" t="s">
         <v>7</v>
@@ -2484,7 +2485,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>85</v>
       </c>
@@ -2498,7 +2499,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>86</v>
       </c>
@@ -2512,7 +2513,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>87</v>
       </c>
@@ -2526,7 +2527,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>88</v>
       </c>
@@ -2540,7 +2541,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>89</v>
       </c>
@@ -2554,7 +2555,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>90</v>
       </c>
@@ -2568,7 +2569,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>91</v>
       </c>
@@ -2582,7 +2583,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>92</v>
       </c>
@@ -2596,7 +2597,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>93</v>
       </c>
@@ -2610,7 +2611,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>94</v>
       </c>
@@ -2624,7 +2625,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>95</v>
       </c>
@@ -2638,7 +2639,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>96</v>
       </c>
@@ -2652,7 +2653,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>97</v>
       </c>
@@ -2666,7 +2667,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>98</v>
       </c>
@@ -2680,7 +2681,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>99</v>
       </c>
@@ -2694,7 +2695,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>112</v>
       </c>
@@ -2708,7 +2709,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>115</v>
       </c>
@@ -2722,7 +2723,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>123</v>
       </c>
@@ -2736,7 +2737,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>124</v>
       </c>
@@ -2750,7 +2751,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>117</v>
       </c>
@@ -2764,7 +2765,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>125</v>
       </c>
@@ -2778,7 +2779,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>121</v>
       </c>
@@ -2792,7 +2793,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>122</v>
       </c>
@@ -2806,7 +2807,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>126</v>
       </c>
@@ -2820,7 +2821,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>127</v>
       </c>
@@ -2834,7 +2835,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>128</v>
       </c>
@@ -2848,7 +2849,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>129</v>
       </c>
@@ -2862,7 +2863,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>130</v>
       </c>
@@ -2877,6 +2878,22 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:D112" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <filters>
+        <filter val="E"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="3">
+      <filters>
+        <filter val="APURÍMAC"/>
+        <filter val="AYACUCHO"/>
+      </filters>
+    </filterColumn>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A15:D84">
+      <sortCondition ref="B1:B112"/>
+    </sortState>
+  </autoFilter>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2894,6 +2911,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="07c8fde6007faf37af3ccef690656753">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1f83a7a0bc9c2dabcf9590cf8de720c" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
@@ -3100,15 +3126,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
   <ds:schemaRefs>
@@ -3121,6 +3138,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97189664-1794-4876-AECF-20AF585E9009}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3137,12 +3162,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica vie 07/08/2026 10:20:10.19
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/02. Encuestas/Insumos limpieza/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="163" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0C6D0910-94C6-426F-A3D0-6267272AD9D5}"/>
+  <xr:revisionPtr revIDLastSave="159" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C896A195-B9B3-4883-8084-FD876F3BB439}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$112</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="141">
   <si>
     <t>CODPER</t>
   </si>
@@ -453,6 +453,12 @@
   </si>
   <si>
     <t>MONICA POZO LOZANO</t>
+  </si>
+  <si>
+    <t>B6</t>
+  </si>
+  <si>
+    <t>ANYELA MILAGROS HUAMAN ROMERO</t>
   </si>
 </sst>
 </file>
@@ -1299,8 +1305,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
-  <dimension ref="A1:D112"/>
+  <dimension ref="A1:D113"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
@@ -1323,7 +1328,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1337,7 +1342,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1351,7 +1356,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1365,7 +1370,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1379,7 +1384,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1393,7 +1398,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1407,7 +1412,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1421,7 +1426,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1435,7 +1440,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1449,7 +1454,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1463,7 +1468,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1477,7 +1482,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1491,7 +1496,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1507,10 +1512,10 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="C15" t="s">
         <v>7</v>
@@ -1521,10 +1526,10 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>66</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>63</v>
+        <v>20</v>
       </c>
       <c r="C16" t="s">
         <v>7</v>
@@ -1535,24 +1540,24 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>65</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>21</v>
       </c>
       <c r="C17" t="s">
         <v>7</v>
       </c>
       <c r="D17" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>68</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>22</v>
       </c>
       <c r="C18" t="s">
         <v>7</v>
@@ -1563,38 +1568,38 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>83</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>94</v>
+        <v>23</v>
       </c>
       <c r="C19" t="s">
         <v>7</v>
       </c>
       <c r="D19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>38</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>43</v>
+        <v>24</v>
       </c>
       <c r="C20" t="s">
         <v>7</v>
       </c>
       <c r="D20" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>71</v>
+        <v>25</v>
       </c>
       <c r="C21" t="s">
         <v>7</v>
@@ -1603,7 +1608,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="22" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1617,7 +1622,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1631,7 +1636,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1645,7 +1650,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1659,7 +1664,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1673,7 +1678,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1687,7 +1692,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1701,7 +1706,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="29" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1715,7 +1720,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1729,7 +1734,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="31" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1743,7 +1748,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1757,7 +1762,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="33" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1771,7 +1776,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="34" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1785,7 +1790,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="35" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1799,7 +1804,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="36" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1813,7 +1818,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="37" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1829,52 +1834,52 @@
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="C38" t="s">
         <v>7</v>
       </c>
       <c r="D38" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="C39" t="s">
         <v>7</v>
       </c>
       <c r="D39" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="C40" t="s">
         <v>7</v>
       </c>
       <c r="D40" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C41" t="s">
         <v>7</v>
@@ -1885,33 +1890,33 @@
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C42" t="s">
         <v>7</v>
       </c>
       <c r="D42" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>21</v>
+        <v>47</v>
       </c>
       <c r="C43" t="s">
         <v>7</v>
       </c>
       <c r="D43" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1925,7 +1930,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="45" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1939,7 +1944,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="46" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1953,7 +1958,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="47" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1967,7 +1972,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="48" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1981,7 +1986,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="49" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1995,7 +2000,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="50" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>50</v>
       </c>
@@ -2009,7 +2014,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="51" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>51</v>
       </c>
@@ -2023,7 +2028,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="52" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>52</v>
       </c>
@@ -2037,7 +2042,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="53" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>53</v>
       </c>
@@ -2051,7 +2056,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="54" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>54</v>
       </c>
@@ -2065,7 +2070,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="55" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>55</v>
       </c>
@@ -2079,7 +2084,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="56" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>56</v>
       </c>
@@ -2093,7 +2098,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="57" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>57</v>
       </c>
@@ -2107,7 +2112,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="58" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>58</v>
       </c>
@@ -2123,19 +2128,19 @@
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A59">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="B59" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="C59" t="s">
         <v>7</v>
       </c>
       <c r="D59" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>60</v>
       </c>
@@ -2149,7 +2154,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="61" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>61</v>
       </c>
@@ -2165,24 +2170,24 @@
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A62">
-        <v>20</v>
+        <v>62</v>
       </c>
       <c r="B62" t="s">
-        <v>25</v>
+        <v>67</v>
       </c>
       <c r="C62" t="s">
         <v>7</v>
       </c>
       <c r="D62" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A63">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="B63" t="s">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="C63" t="s">
         <v>7</v>
@@ -2207,10 +2212,10 @@
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A65">
-        <v>84</v>
+        <v>65</v>
       </c>
       <c r="B65" t="s">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="C65" t="s">
         <v>7</v>
@@ -2221,38 +2226,38 @@
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A66">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="B66" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="C66" t="s">
         <v>7</v>
       </c>
       <c r="D66" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A67">
-        <v>39</v>
+        <v>67</v>
       </c>
       <c r="B67" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="C67" t="s">
         <v>7</v>
       </c>
       <c r="D67" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="68" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A68">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="B68" t="s">
-        <v>23</v>
+        <v>72</v>
       </c>
       <c r="C68" t="s">
         <v>7</v>
@@ -2261,7 +2266,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="69" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>69</v>
       </c>
@@ -2275,7 +2280,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="70" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>70</v>
       </c>
@@ -2289,7 +2294,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="71" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>71</v>
       </c>
@@ -2303,7 +2308,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="72" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>72</v>
       </c>
@@ -2317,7 +2322,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="73" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>73</v>
       </c>
@@ -2331,7 +2336,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="74" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>74</v>
       </c>
@@ -2345,7 +2350,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>75</v>
       </c>
@@ -2359,7 +2364,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="76" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>76</v>
       </c>
@@ -2373,7 +2378,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>77</v>
       </c>
@@ -2387,7 +2392,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="78" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>78</v>
       </c>
@@ -2401,7 +2406,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="79" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>79</v>
       </c>
@@ -2415,7 +2420,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>80</v>
       </c>
@@ -2429,7 +2434,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="81" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>81</v>
       </c>
@@ -2443,7 +2448,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="82" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>82</v>
       </c>
@@ -2459,10 +2464,10 @@
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="B83" t="s">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="C83" t="s">
         <v>7</v>
@@ -2473,10 +2478,10 @@
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84">
-        <v>37</v>
+        <v>84</v>
       </c>
       <c r="B84" t="s">
-        <v>42</v>
+        <v>95</v>
       </c>
       <c r="C84" t="s">
         <v>7</v>
@@ -2485,7 +2490,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="85" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>85</v>
       </c>
@@ -2499,7 +2504,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="86" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>86</v>
       </c>
@@ -2513,7 +2518,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="87" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>87</v>
       </c>
@@ -2527,7 +2532,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="88" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>88</v>
       </c>
@@ -2541,7 +2546,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="89" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>89</v>
       </c>
@@ -2555,7 +2560,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="90" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>90</v>
       </c>
@@ -2569,7 +2574,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="91" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>91</v>
       </c>
@@ -2583,7 +2588,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="92" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>92</v>
       </c>
@@ -2597,7 +2602,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="93" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>93</v>
       </c>
@@ -2611,7 +2616,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="94" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>94</v>
       </c>
@@ -2625,7 +2630,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="95" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>95</v>
       </c>
@@ -2639,7 +2644,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="96" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>96</v>
       </c>
@@ -2653,7 +2658,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="97" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>97</v>
       </c>
@@ -2667,7 +2672,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>98</v>
       </c>
@@ -2681,7 +2686,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="99" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>99</v>
       </c>
@@ -2695,7 +2700,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="100" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>112</v>
       </c>
@@ -2709,7 +2714,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="101" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>115</v>
       </c>
@@ -2723,7 +2728,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="102" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>123</v>
       </c>
@@ -2737,7 +2742,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="103" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>124</v>
       </c>
@@ -2751,7 +2756,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="104" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>117</v>
       </c>
@@ -2765,7 +2770,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="105" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>125</v>
       </c>
@@ -2779,7 +2784,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="106" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>121</v>
       </c>
@@ -2793,7 +2798,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="107" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>122</v>
       </c>
@@ -2807,7 +2812,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="108" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>126</v>
       </c>
@@ -2821,7 +2826,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="109" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>127</v>
       </c>
@@ -2835,7 +2840,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="110" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>128</v>
       </c>
@@ -2849,7 +2854,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="111" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>129</v>
       </c>
@@ -2863,7 +2868,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="112" spans="1:4" hidden="1" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>130</v>
       </c>
@@ -2877,49 +2882,27 @@
         <v>84</v>
       </c>
     </row>
+    <row r="113" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A113" t="s">
+        <v>139</v>
+      </c>
+      <c r="B113" t="s">
+        <v>140</v>
+      </c>
+      <c r="C113" t="s">
+        <v>7</v>
+      </c>
+      <c r="D113" t="s">
+        <v>84</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D112" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="E"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="3">
-      <filters>
-        <filter val="APURÍMAC"/>
-        <filter val="AYACUCHO"/>
-      </filters>
-    </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A15:D84">
-      <sortCondition ref="B1:B112"/>
-    </sortState>
-  </autoFilter>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="07c8fde6007faf37af3ccef690656753">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1f83a7a0bc9c2dabcf9590cf8de720c" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
@@ -3126,26 +3109,27 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97189664-1794-4876-AECF-20AF585E9009}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3162,4 +3146,23 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
+    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica mar 11/08/2026  9:36:48.24
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/02. Encuestas/Insumos limpieza/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="159" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C896A195-B9B3-4883-8084-FD876F3BB439}"/>
+  <xr:revisionPtr revIDLastSave="171" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B480BE2C-FBB4-484E-9F01-23FA5B9F2B71}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="149">
   <si>
     <t>CODPER</t>
   </si>
@@ -459,6 +459,30 @@
   </si>
   <si>
     <t>ANYELA MILAGROS HUAMAN ROMERO</t>
+  </si>
+  <si>
+    <t>B4</t>
+  </si>
+  <si>
+    <t>B5</t>
+  </si>
+  <si>
+    <t>B7</t>
+  </si>
+  <si>
+    <t>B8</t>
+  </si>
+  <si>
+    <t>ANTONIA ESTRADA LAZARO</t>
+  </si>
+  <si>
+    <t>NIMINA HUANSI PISANGO</t>
+  </si>
+  <si>
+    <t>NANCY MAGAN CHAVARRIA</t>
+  </si>
+  <si>
+    <t>SEHILA CAROLINA ALARCON ECHEGARAY</t>
   </si>
 </sst>
 </file>
@@ -1305,7 +1329,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D113"/>
+  <dimension ref="A1:D117"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
@@ -2884,16 +2908,72 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B113" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="C113" t="s">
         <v>7</v>
       </c>
       <c r="D113" t="s">
         <v>84</v>
+      </c>
+    </row>
+    <row r="114" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A114" t="s">
+        <v>142</v>
+      </c>
+      <c r="B114" t="s">
+        <v>146</v>
+      </c>
+      <c r="C114" t="s">
+        <v>7</v>
+      </c>
+      <c r="D114" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="115" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A115" t="s">
+        <v>139</v>
+      </c>
+      <c r="B115" t="s">
+        <v>140</v>
+      </c>
+      <c r="C115" t="s">
+        <v>7</v>
+      </c>
+      <c r="D115" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="116" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A116" t="s">
+        <v>143</v>
+      </c>
+      <c r="B116" t="s">
+        <v>147</v>
+      </c>
+      <c r="C116" t="s">
+        <v>7</v>
+      </c>
+      <c r="D116" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A117" t="s">
+        <v>144</v>
+      </c>
+      <c r="B117" t="s">
+        <v>148</v>
+      </c>
+      <c r="C117" t="s">
+        <v>7</v>
+      </c>
+      <c r="D117" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -2903,6 +2983,17 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="07c8fde6007faf37af3ccef690656753">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1f83a7a0bc9c2dabcf9590cf8de720c" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
@@ -3109,17 +3200,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -3130,6 +3210,17 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
+    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97189664-1794-4876-AECF-20AF585E9009}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3148,17 +3239,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizacion automatica vie 14/08/2026 11:21:31.02
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/02. Encuestas/Insumos limpieza/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="171" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B480BE2C-FBB4-484E-9F01-23FA5B9F2B71}"/>
+  <xr:revisionPtr revIDLastSave="177" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6695CE8D-7F84-4F12-A461-D7AC70117CDE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,9 @@
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$112</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$113</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="151">
   <si>
     <t>CODPER</t>
   </si>
@@ -476,13 +476,19 @@
     <t>ANTONIA ESTRADA LAZARO</t>
   </si>
   <si>
-    <t>NIMINA HUANSI PISANGO</t>
-  </si>
-  <si>
     <t>NANCY MAGAN CHAVARRIA</t>
   </si>
   <si>
     <t>SEHILA CAROLINA ALARCON ECHEGARAY</t>
+  </si>
+  <si>
+    <t>A7</t>
+  </si>
+  <si>
+    <t>JACQUELINE UBILLUS TORRES</t>
+  </si>
+  <si>
+    <t>NIMIA HUANSI PISANGO</t>
   </si>
 </sst>
 </file>
@@ -1329,7 +1335,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D117"/>
+  <dimension ref="A1:D118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
@@ -2824,27 +2830,27 @@
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>122</v>
+        <v>148</v>
       </c>
       <c r="B107" t="s">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="C107" t="s">
         <v>5</v>
       </c>
       <c r="D107" t="s">
-        <v>84</v>
+        <v>102</v>
       </c>
     </row>
     <row r="108" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="B108" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="C108" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D108" t="s">
         <v>84</v>
@@ -2852,10 +2858,10 @@
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B109" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C109" t="s">
         <v>7</v>
@@ -2866,10 +2872,10 @@
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B110" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C110" t="s">
         <v>7</v>
@@ -2880,10 +2886,10 @@
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B111" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C111" t="s">
         <v>7</v>
@@ -2894,10 +2900,10 @@
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B112" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C112" t="s">
         <v>7</v>
@@ -2908,10 +2914,10 @@
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
       <c r="B113" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="C113" t="s">
         <v>7</v>
@@ -2922,10 +2928,10 @@
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B114" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C114" t="s">
         <v>7</v>
@@ -2936,10 +2942,10 @@
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B115" t="s">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="C115" t="s">
         <v>7</v>
@@ -2950,29 +2956,43 @@
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="B116" t="s">
-        <v>147</v>
+        <v>140</v>
       </c>
       <c r="C116" t="s">
         <v>7</v>
       </c>
       <c r="D116" t="s">
-        <v>102</v>
+        <v>84</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
+        <v>143</v>
+      </c>
+      <c r="B117" t="s">
+        <v>146</v>
+      </c>
+      <c r="C117" t="s">
+        <v>7</v>
+      </c>
+      <c r="D117" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="118" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A118" t="s">
         <v>144</v>
       </c>
-      <c r="B117" t="s">
-        <v>148</v>
-      </c>
-      <c r="C117" t="s">
-        <v>7</v>
-      </c>
-      <c r="D117" t="s">
+      <c r="B118" t="s">
+        <v>147</v>
+      </c>
+      <c r="C118" t="s">
+        <v>7</v>
+      </c>
+      <c r="D118" t="s">
         <v>102</v>
       </c>
     </row>
@@ -2983,14 +3003,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3201,21 +3219,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3240,9 +3257,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
+    <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Actualizacion automatica lun 17/08/2026 11:05:57.01
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/02. Encuestas/Insumos limpieza/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="177" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6695CE8D-7F84-4F12-A461-D7AC70117CDE}"/>
+  <xr:revisionPtr revIDLastSave="185" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{442B2AD3-42FB-40F2-A3F2-7CA2F9CF6AD1}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$113</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$118</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -2153,7 +2153,7 @@
         <v>7</v>
       </c>
       <c r="D58" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.3">
@@ -3003,15 +3003,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="07c8fde6007faf37af3ccef690656753">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1f83a7a0bc9c2dabcf9590cf8de720c" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
@@ -3218,6 +3209,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3230,14 +3230,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97189664-1794-4876-AECF-20AF585E9009}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3256,6 +3248,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizacion automatica mié 19/08/2026  9:17:20.30
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/02. Encuestas/Insumos limpieza/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="185" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{442B2AD3-42FB-40F2-A3F2-7CA2F9CF6AD1}"/>
+  <xr:revisionPtr revIDLastSave="194" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F6DBE21-3E1C-4BFA-8219-AC95A371D142}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="152">
   <si>
     <t>CODPER</t>
   </si>
@@ -489,6 +489,9 @@
   </si>
   <si>
     <t>NIMIA HUANSI PISANGO</t>
+  </si>
+  <si>
+    <t>REASIGNACION</t>
   </si>
 </sst>
 </file>
@@ -1335,16 +1338,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D118"/>
+  <dimension ref="A1:E118"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="58.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="38.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1357,8 +1361,11 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1372,7 +1379,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1386,7 +1393,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1400,7 +1407,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1414,7 +1421,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1428,7 +1435,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1442,7 +1449,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1456,7 +1463,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1470,7 +1477,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1484,7 +1491,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -1498,7 +1505,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -1512,7 +1519,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -1526,7 +1533,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -1540,7 +1547,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1554,7 +1561,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1568,7 +1575,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1582,7 +1589,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1596,7 +1603,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1610,7 +1617,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1624,7 +1631,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1638,7 +1645,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1652,7 +1659,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1666,7 +1673,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1680,7 +1687,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1694,7 +1701,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1708,7 +1715,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1722,7 +1729,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1735,8 +1742,11 @@
       <c r="D28" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E28" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1750,7 +1760,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1764,7 +1774,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1778,7 +1788,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -2688,7 +2698,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>97</v>
       </c>
@@ -2702,7 +2712,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>98</v>
       </c>
@@ -2716,7 +2726,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="99" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>99</v>
       </c>
@@ -2730,7 +2740,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="100" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>112</v>
       </c>
@@ -2743,8 +2753,11 @@
       <c r="D100" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="101" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E100" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>115</v>
       </c>
@@ -2758,7 +2771,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="102" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>123</v>
       </c>
@@ -2772,7 +2785,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="103" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>124</v>
       </c>
@@ -2786,7 +2799,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="104" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>117</v>
       </c>
@@ -2800,7 +2813,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="105" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>125</v>
       </c>
@@ -2814,7 +2827,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="106" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>121</v>
       </c>
@@ -2828,7 +2841,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="107" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>148</v>
       </c>
@@ -2842,7 +2855,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="108" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>122</v>
       </c>
@@ -2856,7 +2869,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="109" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>126</v>
       </c>
@@ -2870,7 +2883,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="110" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>127</v>
       </c>
@@ -2884,7 +2897,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="111" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>128</v>
       </c>
@@ -2898,7 +2911,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="112" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>129</v>
       </c>
@@ -3003,6 +3016,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="07c8fde6007faf37af3ccef690656753">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1f83a7a0bc9c2dabcf9590cf8de720c" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
@@ -3209,15 +3231,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3230,6 +3243,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97189664-1794-4876-AECF-20AF585E9009}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3248,14 +3269,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizacion automatica mié 19/08/2026  9:41:05.03
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="194" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F6DBE21-3E1C-4BFA-8219-AC95A371D142}"/>
+  <xr:revisionPtr revIDLastSave="202" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BCFC98D-E238-4F9F-AE8D-62B7F5A7093B}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$D$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$E$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="152">
   <si>
     <t>CODPER</t>
   </si>
@@ -1345,7 +1345,7 @@
     <col min="2" max="2" width="58.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="4.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="38.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -2723,6 +2723,9 @@
         <v>7</v>
       </c>
       <c r="D98" t="s">
+        <v>102</v>
+      </c>
+      <c r="E98" t="s">
         <v>84</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizacion automatica lun 24/08/2026  8:37:43.90
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="202" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BCFC98D-E238-4F9F-AE8D-62B7F5A7093B}"/>
+  <xr:revisionPtr revIDLastSave="205" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE75F371-D93B-4F66-B551-7C62BC5838B8}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$E$118</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -3019,15 +3019,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="07c8fde6007faf37af3ccef690656753">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1f83a7a0bc9c2dabcf9590cf8de720c" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
@@ -3234,6 +3225,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3246,14 +3246,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97189664-1794-4876-AECF-20AF585E9009}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3272,6 +3264,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizacion automatica vie 28/08/2026  9:10:29.50
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/02. Encuestas/Insumos limpieza/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="205" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BE75F371-D93B-4F66-B551-7C62BC5838B8}"/>
+  <xr:revisionPtr revIDLastSave="204" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E515086-C2CB-43E2-A83B-2D3FEF97E09C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="378" uniqueCount="152">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="154">
   <si>
     <t>CODPER</t>
   </si>
@@ -492,6 +492,12 @@
   </si>
   <si>
     <t>REASIGNACION</t>
+  </si>
+  <si>
+    <t>B9</t>
+  </si>
+  <si>
+    <t>SAGRARIO MAGNOLIA ORTIZ MOLLEPAZA</t>
   </si>
 </sst>
 </file>
@@ -1338,7 +1344,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E118"/>
+  <dimension ref="A1:E119"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
@@ -3012,6 +3018,20 @@
         <v>102</v>
       </c>
     </row>
+    <row r="119" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
+        <v>152</v>
+      </c>
+      <c r="B119" t="s">
+        <v>153</v>
+      </c>
+      <c r="C119" t="s">
+        <v>7</v>
+      </c>
+      <c r="D119" t="s">
+        <v>79</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="18" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3019,6 +3039,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="07c8fde6007faf37af3ccef690656753">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1f83a7a0bc9c2dabcf9590cf8de720c" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
@@ -3225,15 +3254,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3246,6 +3266,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97189664-1794-4876-AECF-20AF585E9009}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3264,14 +3292,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizacion automatica lun 31/08/2026  8:41:50.13
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/02. Encuestas/Insumos limpieza/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="204" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3E515086-C2CB-43E2-A83B-2D3FEF97E09C}"/>
+  <xr:revisionPtr revIDLastSave="208" documentId="8_{BBF476B9-BDC2-4635-8D81-92938E401460}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AC9F634-05C2-4023-8517-EC05A7FFB6EE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$E$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$E$119</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="154">
   <si>
     <t>CODPER</t>
   </si>
@@ -2256,7 +2256,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>65</v>
       </c>
@@ -2270,7 +2270,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>66</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>67</v>
       </c>
@@ -2298,7 +2298,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>68</v>
       </c>
@@ -2312,7 +2312,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>69</v>
       </c>
@@ -2326,7 +2326,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>70</v>
       </c>
@@ -2339,8 +2339,11 @@
       <c r="D70" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E70" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>71</v>
       </c>
@@ -2354,7 +2357,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>72</v>
       </c>
@@ -2368,7 +2371,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>73</v>
       </c>
@@ -2382,7 +2385,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>74</v>
       </c>
@@ -2396,7 +2399,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>75</v>
       </c>
@@ -2410,7 +2413,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>76</v>
       </c>
@@ -2424,7 +2427,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>77</v>
       </c>
@@ -2438,7 +2441,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>78</v>
       </c>
@@ -2452,7 +2455,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>79</v>
       </c>
@@ -2466,7 +2469,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>80</v>
       </c>
@@ -3039,15 +3042,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101007183A11C1BA9EC45BAE4956AD7AAC49F" ma:contentTypeVersion="13" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="07c8fde6007faf37af3ccef690656753">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="667d70cb-f49f-4223-87b6-a8a0e4fc3231" xmlns:ns3="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a1f83a7a0bc9c2dabcf9590cf8de720c" ns2:_="" ns3:_="">
     <xsd:import namespace="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
@@ -3254,6 +3248,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3266,14 +3269,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97189664-1794-4876-AECF-20AF585E9009}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3292,6 +3287,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76243D71-2718-4643-8B37-CE87F4587C9C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED8B7C50-84DD-4E30-997A-3C61B4A70484}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Actualizacion automatica jue 10/09/2026 11:54:01.17
</commit_message>
<xml_diff>
--- a/data/BD Personal.xlsx
+++ b/data/BD Personal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://apoyoconsultoria0.sharepoint.com/sites/fileserver/Polticas Pblicas/6 Proyectos/2025/2025-070-O IJM - Linea de base/04. Analisis/03. Programacion/06. Dashboard Seguimiento Web/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E01492CD-3A7D-4144-89DC-97B8968C6F4E}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="11_A10BAE44CD785D61F5141092B1107384533E0B90" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{78D69169-60F1-420D-BB87-B4C6C30E1148}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Exported" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$F$119</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Exported!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="390" uniqueCount="157">
   <si>
     <t>CODPER</t>
   </si>
@@ -501,6 +501,12 @@
   </si>
   <si>
     <t>SAGRARIO MAGNOLIA ORTIZ MOLLEPAZA</t>
+  </si>
+  <si>
+    <t>C1</t>
+  </si>
+  <si>
+    <t>JENNY SALON ANAHUA</t>
   </si>
 </sst>
 </file>
@@ -508,7 +514,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -539,9 +545,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -856,7 +863,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F119"/>
+  <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.109375" bestFit="1" customWidth="1"/>
@@ -1109,6 +1116,12 @@
       <c r="D17" t="s">
         <v>23</v>
       </c>
+      <c r="E17" t="s">
+        <v>39</v>
+      </c>
+      <c r="F17" s="2">
+        <v>46252</v>
+      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18">
@@ -1829,6 +1842,12 @@
       <c r="D68" t="s">
         <v>23</v>
       </c>
+      <c r="E68" t="s">
+        <v>39</v>
+      </c>
+      <c r="F68" s="2">
+        <v>46252</v>
+      </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69">
@@ -2560,6 +2579,20 @@
       </c>
       <c r="D119" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="120" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
+        <v>155</v>
+      </c>
+      <c r="B120" t="s">
+        <v>156</v>
+      </c>
+      <c r="C120" t="s">
+        <v>10</v>
+      </c>
+      <c r="D120" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -2568,6 +2601,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="667d70cb-f49f-4223-87b6-a8a0e4fc3231">
@@ -2576,15 +2618,6 @@
     <TaxCatchAll xmlns="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2795,20 +2828,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E73E3A5A-F8DC-40E4-A1F8-9A051C36DEF4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="667d70cb-f49f-4223-87b6-a8a0e4fc3231"/>
     <ds:schemaRef ds:uri="c37f41b3-fada-4b69-b314-7ed8c2ce1ec6"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{630299A7-E824-4D69-AA5E-3193E7062408}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>